<commit_message>
Auto update master.json, manifests, and repo contents
</commit_message>
<xml_diff>
--- a/master.xlsx
+++ b/master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fengbo/GitHub/soseki-manuscripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2047FAAD-18CB-4B46-A836-70E9576B1F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2558FD9A-0011-9147-AC24-1172959DB71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16040" yWindow="620" windowWidth="15960" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2431,7 +2431,7 @@
     <t>https://scholarbo.github.io/soseki-manuscripts/manifests/manifest-216-w01.json</t>
   </si>
   <si>
-    <t>『時運』</t>
+    <t>『時運』a</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>

</xml_diff>